<commit_message>
Add executive capture deploy: Docker, Render blueprint, health check, Pages config.
Wire digi.html to POST only; serve API via gunicorn container. Append-only
Submission log commits to GitHub when token is set. Document Render setup.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/Merrakii_Business_Capture.xlsx
+++ b/docs/Merrakii_Business_Capture.xlsx
@@ -7,13 +7,14 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Company content" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Brand and contact" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Human support" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Payment gateway" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Legal and consent" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Programs and partners" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Operations handoff" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Submission log" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Company content" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Brand and contact" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Human support" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Payment gateway" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Legal and consent" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Programs and partners" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Operations handoff" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -434,6 +435,79 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="4" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Timestamp (UTC)</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Q#</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Question</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Response</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-04-26T11:48:13Z</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Company content</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>What short tagline or one-line value proposition should appear with the Merrakii brand on the home or landing experience?</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Test answer from curl</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -471,7 +545,7 @@
           <t>What short tagline or one-line value proposition should appear with the Merrakii brand on the home or landing experience?</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n"/>
+      <c r="B3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -550,7 +624,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -664,7 +738,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -794,7 +868,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -956,7 +1030,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1094,7 +1168,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1208,7 +1282,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
chore(executive-inputs): append submission 2026-04-27T14:14:43.280977+00:00
</commit_message>
<xml_diff>
--- a/docs/Merrakii_Business_Capture.xlsx
+++ b/docs/Merrakii_Business_Capture.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -494,6 +494,31 @@
       <c r="E2" t="inlineStr">
         <is>
           <t>Test answer from curl</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-04-27T14:14:43Z</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Company content</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>What short tagline or one-line value proposition should appear with the Merrakii brand on the home or landing experience?</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>abcd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(executive-inputs): append submission 2026-04-27T14:18:36.929708+00:00
</commit_message>
<xml_diff>
--- a/docs/Merrakii_Business_Capture.xlsx
+++ b/docs/Merrakii_Business_Capture.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -519,6 +519,31 @@
       <c r="E3" t="inlineStr">
         <is>
           <t>abcd</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-04-27T14:18:36Z</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Company content</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>What short tagline or one-line value proposition should appear with the Merrakii brand on the home or landing experience?</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>qqqq</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(executive-inputs): upsert submission 2026-04-27T15:04:17.339995+00:00
</commit_message>
<xml_diff>
--- a/docs/Merrakii_Business_Capture.xlsx
+++ b/docs/Merrakii_Business_Capture.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -475,7 +475,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-26T11:48:13Z</t>
+          <t>2026-04-27T15:04:17Z</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -493,57 +493,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Test answer from curl</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-04-27T14:14:43Z</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Company content</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>What short tagline or one-line value proposition should appear with the Merrakii brand on the home or landing experience?</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>abcd</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-04-27T14:18:36Z</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Company content</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>What short tagline or one-line value proposition should appear with the Merrakii brand on the home or landing experience?</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>qqqq</t>
+          <t>wwww</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(executive-inputs): upsert submission 2026-04-27T15:05:04.951930+00:00
</commit_message>
<xml_diff>
--- a/docs/Merrakii_Business_Capture.xlsx
+++ b/docs/Merrakii_Business_Capture.xlsx
@@ -475,7 +475,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-27T15:04:17Z</t>
+          <t>2026-04-27T15:05:04Z</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -493,7 +493,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>wwww</t>
+          <t>eeee</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(executive-inputs): upsert submission 2026-04-27T15:06:10.639629+00:00
</commit_message>
<xml_diff>
--- a/docs/Merrakii_Business_Capture.xlsx
+++ b/docs/Merrakii_Business_Capture.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -475,7 +475,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-27T15:05:04Z</t>
+          <t>2026-04-27T15:06:10Z</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -494,6 +494,31 @@
       <c r="E2" t="inlineStr">
         <is>
           <t>eeee</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-04-27T15:06:10Z</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Company content</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>What ‘About Merrakii’ narrative should students read (mission, years in business, geography served)? Prefer word count or bullet limit if you have one.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>bgbgbgbgb</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(executive-inputs): upsert submission 2026-04-27T15:07:08.997162+00:00
</commit_message>
<xml_diff>
--- a/docs/Merrakii_Business_Capture.xlsx
+++ b/docs/Merrakii_Business_Capture.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -475,7 +475,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-27T15:06:10Z</t>
+          <t>2026-04-27T15:07:08Z</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -500,7 +500,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-27T15:06:10Z</t>
+          <t>2026-04-27T15:07:08Z</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -519,6 +519,31 @@
       <c r="E3" t="inlineStr">
         <is>
           <t>bgbgbgbgb</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-04-27T15:07:08Z</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Legal and consent</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>9</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>For document uploads (ID, marksheets): what declaration must the user confirm (authenticity, purpose)?</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>fjfjfj</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(executive-inputs): upsert submission 2026-04-27T15:07:48.912015+00:00
</commit_message>
<xml_diff>
--- a/docs/Merrakii_Business_Capture.xlsx
+++ b/docs/Merrakii_Business_Capture.xlsx
@@ -475,7 +475,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-27T15:07:08Z</t>
+          <t>2026-04-27T15:07:48Z</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -491,16 +491,12 @@
           <t>What short tagline or one-line value proposition should appear with the Merrakii brand on the home or landing experience?</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>eeee</t>
-        </is>
-      </c>
+      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-27T15:07:08Z</t>
+          <t>2026-04-27T15:07:48Z</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -516,16 +512,12 @@
           <t>What ‘About Merrakii’ narrative should students read (mission, years in business, geography served)? Prefer word count or bullet limit if you have one.</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>bgbgbgbgb</t>
-        </is>
-      </c>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-27T15:07:08Z</t>
+          <t>2026-04-27T15:07:48Z</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -541,11 +533,7 @@
           <t>For document uploads (ID, marksheets): what declaration must the user confirm (authenticity, purpose)?</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>fjfjfj</t>
-        </is>
-      </c>
+      <c r="E4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(executive-inputs): upsert submission 2026-04-27T15:10:20.009323+00:00
</commit_message>
<xml_diff>
--- a/docs/Merrakii_Business_Capture.xlsx
+++ b/docs/Merrakii_Business_Capture.xlsx
@@ -475,7 +475,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-27T15:07:48Z</t>
+          <t>2026-04-27T15:10:19Z</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -491,7 +491,11 @@
           <t>What short tagline or one-line value proposition should appear with the Merrakii brand on the home or landing experience?</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Merrakii</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -512,7 +516,6 @@
           <t>What ‘About Merrakii’ narrative should students read (mission, years in business, geography served)? Prefer word count or bullet limit if you have one.</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -533,7 +536,6 @@
           <t>For document uploads (ID, marksheets): what declaration must the user confirm (authenticity, purpose)?</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(executive-inputs): upsert submission 2026-04-28T05:02:55.618286+00:00
</commit_message>
<xml_diff>
--- a/docs/Merrakii_Business_Capture.xlsx
+++ b/docs/Merrakii_Business_Capture.xlsx
@@ -475,7 +475,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-27T15:10:19Z</t>
+          <t>2026-04-28T05:02:55Z</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -493,14 +493,14 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Merrakii</t>
+          <t>qwert</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-27T15:07:48Z</t>
+          <t>2026-04-28T05:02:55Z</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -516,11 +516,12 @@
           <t>What ‘About Merrakii’ narrative should students read (mission, years in business, geography served)? Prefer word count or bullet limit if you have one.</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-27T15:07:48Z</t>
+          <t>2026-04-28T05:02:55Z</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -536,6 +537,7 @@
           <t>For document uploads (ID, marksheets): what declaration must the user confirm (authenticity, purpose)?</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(executive-inputs): upsert submission 2026-04-28T05:07:12.166257+00:00
</commit_message>
<xml_diff>
--- a/docs/Merrakii_Business_Capture.xlsx
+++ b/docs/Merrakii_Business_Capture.xlsx
@@ -475,7 +475,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-28T05:02:55Z</t>
+          <t>2026-04-28T05:07:11Z</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -491,16 +491,12 @@
           <t>What short tagline or one-line value proposition should appear with the Merrakii brand on the home or landing experience?</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>qwert</t>
-        </is>
-      </c>
+      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-28T05:02:55Z</t>
+          <t>2026-04-28T05:07:11Z</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -521,7 +517,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-28T05:02:55Z</t>
+          <t>2026-04-28T05:07:11Z</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">

</xml_diff>

<commit_message>
chore(executive-inputs): upsert submission 2026-04-29T11:22:02.742825+00:00
</commit_message>
<xml_diff>
--- a/docs/Merrakii_Business_Capture.xlsx
+++ b/docs/Merrakii_Business_Capture.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -491,12 +491,11 @@
           <t>What short tagline or one-line value proposition should appear with the Merrakii brand on the home or landing experience?</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-28T05:07:11Z</t>
+          <t>2026-04-29T11:22:02Z</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -512,7 +511,11 @@
           <t>What ‘About Merrakii’ narrative should students read (mission, years in business, geography served)? Prefer word count or bullet limit if you have one.</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>"About Us" section exists in the current website</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -533,7 +536,106 @@
           <t>For document uploads (ID, marksheets): what declaration must the user confirm (authenticity, purpose)?</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-04-29T11:22:02Z</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Company content</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>List any factual claims we may display (e.g. number of students counselled, partner institutes, success stories)—and confirm each is accurate and approved for marketing.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>This could come in later once we establish some credibility.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-04-29T11:22:02Z</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Company content</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Do you want an ‘Our team’ or counsellor profile section? If yes, provide names, roles, photos, and bios—or confirm ‘no’.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-04-29T11:22:02Z</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Company content</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>7</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Do you want to show office photos or a virtual tour link? Provide assets or URLs.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-04-29T11:22:02Z</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Company content</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>9</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>What languages should customer-facing marketing copy use at launch (e.g. English only, English + Hindi)?</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(executive-inputs): upsert submission 2026-04-30T10:09:54.389940+00:00
</commit_message>
<xml_diff>
--- a/docs/Merrakii_Business_Capture.xlsx
+++ b/docs/Merrakii_Business_Capture.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -475,7 +475,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-28T05:07:11Z</t>
+          <t>2026-04-30T10:09:54Z</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -491,11 +491,16 @@
           <t>What short tagline or one-line value proposition should appear with the Merrakii brand on the home or landing experience?</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>We already have the website in place, which does not carry any tagline at present.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-29T11:22:02Z</t>
+          <t>2026-04-30T10:09:54Z</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -540,7 +545,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-29T11:22:02Z</t>
+          <t>2026-04-30T10:09:54Z</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -565,7 +570,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-04-29T11:22:02Z</t>
+          <t>2026-04-30T10:09:54Z</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -590,7 +595,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-29T11:22:02Z</t>
+          <t>2026-04-30T10:09:54Z</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -615,7 +620,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-29T11:22:02Z</t>
+          <t>2026-04-30T10:09:54Z</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -634,6 +639,571 @@
       <c r="E8" t="inlineStr">
         <is>
           <t>English</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-04-30T10:09:54Z</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Company content</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>What differentiators should we emphasise versus generic ed-tech (e.g. offline office, counsellor-led, exam prep + admissions)?</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>“A transparent platform to discover, compare, and enroll in India’s top entrance prep institutes."
+(We can also add an educational service platform)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-04-30T10:09:54Z</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Company content</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>May we name specific institutes or exams as ‘partners’ or ‘we help with’ on the site? If yes, list exact wording Merrakii approves; if no, say so.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04-30T10:09:54Z</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Company content</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>8</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Do you have student testimonials Merrakii authorises for the app? Provide quote text, first name or initials, and written permission where required.</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>This would come later, once we have students who have successfully enrolled in different institutes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-04-30T10:09:54Z</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Brand and contact</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>What is the legal registered name of the entity that owns the business (for receipts and legal footers)?</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>MUNJAL UNIVERSAL CONSULTANCY PVT LTD</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-04-30T10:09:54Z</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Brand and contact</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>What customer-facing brand name must appear if it differs from the legal name?</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>MERRAKII is the brand identity</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-04-30T10:09:54Z</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Brand and contact</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Provide logo files (master formats you have) and primary/secondary brand colours for the app shell.</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>I shall provide them in a separate mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-04-30T10:09:54Z</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Brand and contact</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>What is the main office address to show (street, city, state, PIN)—for ‘Visit us’ or contact page?</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>T-14
+Salcon Rasvilas
+Saket District Centre
+Saket
+New Delhi - 17</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-04-30T10:09:54Z</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Brand and contact</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>5</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>What is the main public email for inquiries (e.g. hello@…)?</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">info@merrakii.co.in
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-04-30T10:09:54Z</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Brand and contact</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>6</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>What phone number(s) should appear for general inquiries? Label each (e.g. admissions, billing) if different.</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>8800838055 - Admissions
+9899099710 - Admissions
+9319001573 - Billing</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-04-30T10:09:54Z</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Brand and contact</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>7</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>What are Merrakii’s official website and social profile URLs (Instagram, LinkedIn, YouTube, etc.) to link from the app?</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">www.merrakii.co.in
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-04-30T10:09:54Z</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Brand and contact</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>8</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>What are regular business hours for the office and for phone support (timezone included)?</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>10 am - 6pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-04-30T10:09:54Z</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Brand and contact</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>9</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Should we display a map link (Google Maps) for the office? If yes, provide the URL or coordinates.</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>already there on the website</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-04-30T10:09:54Z</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Human support</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>When a student needs human help during search or application, what is the primary phone number to call?</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>8800838055 - Admissions
+9899099710 - Admissions</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-04-30T10:09:54Z</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Human support</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Is that number the same for post-enrollment questions (fees, documents) or different? List each number and purpose.</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-04-30T10:09:54Z</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Human support</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>3</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Are calls toll-free, standard STD, or WhatsApp voice? Specify.</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Standard
+whats app</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-04-30T10:09:54Z</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Human support</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>4</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>What hours is live phone support staffed? What should we tell users outside those hours (e.g. leave SMS, callback)?</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>10am - 6pm
+call back, leave sms</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-04-30T10:09:54Z</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Human support</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>5</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Do you offer WhatsApp chat for support? If yes, provide the business number and any welcome message Merrakii wants.</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>We would want the human support to come in through whats app and even AI Intervention through chat bots etc</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-04-30T10:09:54Z</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Human support</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>6</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Do you offer email ticketing only for certain topics? List topic → email address.</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Not as of now, but we would want this feature.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-04-30T10:09:54Z</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Human support</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>7</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Do you want an in-app ‘Request a counsellor callback’ flow? If yes, what fields may we collect (name, phone, preferred time)?</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes, we want this.
+Name, Phone, time </t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-04-30T10:09:54Z</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Human support</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>8</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>What is the maximum callback commitment Merrakii wants displayed (e.g. within 24 business hours)?</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>within 24 business hours</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-04-30T10:09:54Z</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Human support</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>9</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>For escalations (payment failed, document rejected), who is the internal role name students hear (e.g. ‘admissions desk’)—not personal names unless required?</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Admissions Desk
+May we help you
+etc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-04-30T10:09:54Z</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Human support</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>10</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Should we show the physical office as an option (‘Visit us for in-person counselling’)? If yes, confirm address and whether appointment is required.</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Yes, Same as the address mentioned</t>
         </is>
       </c>
     </row>

</xml_diff>